<commit_message>
feat: implement comprehensive visitor management system with admin analytics, gate console, and multi-category pass generation workflows
</commit_message>
<xml_diff>
--- a/backend/Community_Testing_Credentials_v2.xlsx
+++ b/backend/Community_Testing_Credentials_v2.xlsx
@@ -4924,7 +4924,7 @@
         <v>Apartment</v>
       </c>
       <c r="D12">
-        <v>750</v>
+        <v>1050</v>
       </c>
       <c r="E12" t="str">
         <v>Occupied</v>
@@ -4964,7 +4964,7 @@
         <v>Apartment</v>
       </c>
       <c r="D14">
-        <v>900</v>
+        <v>750</v>
       </c>
       <c r="E14" t="str">
         <v>Occupied</v>
@@ -4984,7 +4984,7 @@
         <v>Apartment</v>
       </c>
       <c r="D15">
-        <v>900</v>
+        <v>750</v>
       </c>
       <c r="E15" t="str">
         <v>Occupied</v>
@@ -5004,7 +5004,7 @@
         <v>Apartment</v>
       </c>
       <c r="D16">
-        <v>1050</v>
+        <v>900</v>
       </c>
       <c r="E16" t="str">
         <v>Occupied</v>
@@ -5024,7 +5024,7 @@
         <v>Apartment</v>
       </c>
       <c r="D17">
-        <v>1050</v>
+        <v>750</v>
       </c>
       <c r="E17" t="str">
         <v>Occupied</v>
@@ -5044,7 +5044,7 @@
         <v>Apartment</v>
       </c>
       <c r="D18">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="E18" t="str">
         <v>Occupied</v>
@@ -5064,7 +5064,7 @@
         <v>Apartment</v>
       </c>
       <c r="D19">
-        <v>1050</v>
+        <v>900</v>
       </c>
       <c r="E19" t="str">
         <v>Occupied</v>
@@ -5084,7 +5084,7 @@
         <v>Apartment</v>
       </c>
       <c r="D20">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="E20" t="str">
         <v>Occupied</v>
@@ -5124,7 +5124,7 @@
         <v>Apartment</v>
       </c>
       <c r="D22">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="E22" t="str">
         <v>Occupied</v>
@@ -5144,7 +5144,7 @@
         <v>Apartment</v>
       </c>
       <c r="D23">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="E23" t="str">
         <v>Occupied</v>
@@ -5184,7 +5184,7 @@
         <v>Apartment</v>
       </c>
       <c r="D25">
-        <v>750</v>
+        <v>1050</v>
       </c>
       <c r="E25" t="str">
         <v>Occupied</v>
@@ -5224,7 +5224,7 @@
         <v>Apartment</v>
       </c>
       <c r="D27">
-        <v>900</v>
+        <v>1050</v>
       </c>
       <c r="E27" t="str">
         <v>Occupied</v>
@@ -5244,7 +5244,7 @@
         <v>Apartment</v>
       </c>
       <c r="D28">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="E28" t="str">
         <v>Occupied</v>
@@ -5264,7 +5264,7 @@
         <v>Apartment</v>
       </c>
       <c r="D29">
-        <v>900</v>
+        <v>1050</v>
       </c>
       <c r="E29" t="str">
         <v>Occupied</v>
@@ -5304,7 +5304,7 @@
         <v>Apartment</v>
       </c>
       <c r="D31">
-        <v>1050</v>
+        <v>900</v>
       </c>
       <c r="E31" t="str">
         <v>Occupied</v>
@@ -5344,7 +5344,7 @@
         <v>Apartment</v>
       </c>
       <c r="D33">
-        <v>750</v>
+        <v>1050</v>
       </c>
       <c r="E33" t="str">
         <v>Occupied</v>
@@ -5384,7 +5384,7 @@
         <v>Apartment</v>
       </c>
       <c r="D35">
-        <v>750</v>
+        <v>1050</v>
       </c>
       <c r="E35" t="str">
         <v>Occupied</v>
@@ -5404,7 +5404,7 @@
         <v>Apartment</v>
       </c>
       <c r="D36">
-        <v>1050</v>
+        <v>900</v>
       </c>
       <c r="E36" t="str">
         <v>Occupied</v>
@@ -5424,7 +5424,7 @@
         <v>Villa</v>
       </c>
       <c r="D37">
-        <v>2000</v>
+        <v>1800</v>
       </c>
       <c r="E37" t="str">
         <v>Occupied</v>
@@ -5444,7 +5444,7 @@
         <v>Villa</v>
       </c>
       <c r="D38">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="E38" t="str">
         <v>Occupied</v>
@@ -5464,7 +5464,7 @@
         <v>Villa</v>
       </c>
       <c r="D39">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E39" t="str">
         <v>Occupied</v>
@@ -5484,7 +5484,7 @@
         <v>Villa</v>
       </c>
       <c r="D40">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E40" t="str">
         <v>Occupied</v>
@@ -5524,7 +5524,7 @@
         <v>Villa</v>
       </c>
       <c r="D42">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E42" t="str">
         <v>Occupied</v>
@@ -5644,7 +5644,7 @@
         <v>Villa</v>
       </c>
       <c r="D48">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="E48" t="str">
         <v>Occupied</v>
@@ -5664,7 +5664,7 @@
         <v>Villa</v>
       </c>
       <c r="D49">
-        <v>2000</v>
+        <v>1800</v>
       </c>
       <c r="E49" t="str">
         <v>Occupied</v>
@@ -5684,7 +5684,7 @@
         <v>Villa</v>
       </c>
       <c r="D50">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="E50" t="str">
         <v>Occupied</v>
@@ -5724,7 +5724,7 @@
         <v>Villa</v>
       </c>
       <c r="D52">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E52" t="str">
         <v>Occupied</v>
@@ -5744,7 +5744,7 @@
         <v>Villa</v>
       </c>
       <c r="D53">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E53" t="str">
         <v>Occupied</v>
@@ -5784,7 +5784,7 @@
         <v>Villa</v>
       </c>
       <c r="D55">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E55" t="str">
         <v>Occupied</v>
@@ -5804,7 +5804,7 @@
         <v>Villa</v>
       </c>
       <c r="D56">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E56" t="str">
         <v>Occupied</v>
@@ -5844,7 +5844,7 @@
         <v>Villa</v>
       </c>
       <c r="D58">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E58" t="str">
         <v>Vacant</v>
@@ -5904,7 +5904,7 @@
         <v>Villa</v>
       </c>
       <c r="D61">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="E61" t="str">
         <v>Vacant</v>
@@ -5924,7 +5924,7 @@
         <v>Villa</v>
       </c>
       <c r="D62">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E62" t="str">
         <v>Vacant</v>
@@ -5944,7 +5944,7 @@
         <v>Villa</v>
       </c>
       <c r="D63">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E63" t="str">
         <v>Vacant</v>
@@ -5964,7 +5964,7 @@
         <v>Villa</v>
       </c>
       <c r="D64">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E64" t="str">
         <v>Vacant</v>
@@ -5984,7 +5984,7 @@
         <v>Villa</v>
       </c>
       <c r="D65">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E65" t="str">
         <v>Vacant</v>
@@ -6004,7 +6004,7 @@
         <v>Villa</v>
       </c>
       <c r="D66">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="E66" t="str">
         <v>Vacant</v>
@@ -6024,7 +6024,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D67">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="E67" t="str">
         <v>Occupied</v>
@@ -6064,7 +6064,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D69">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E69" t="str">
         <v>Occupied</v>
@@ -6084,7 +6084,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D70">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E70" t="str">
         <v>Occupied</v>
@@ -6104,7 +6104,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D71">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E71" t="str">
         <v>Occupied</v>
@@ -6144,7 +6144,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D73">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E73" t="str">
         <v>Occupied</v>
@@ -6164,7 +6164,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D74">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="E74" t="str">
         <v>Occupied</v>
@@ -6184,7 +6184,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D75">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="E75" t="str">
         <v>Occupied</v>
@@ -6204,7 +6204,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D76">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E76" t="str">
         <v>Occupied</v>
@@ -6224,7 +6224,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D77">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E77" t="str">
         <v>Occupied</v>
@@ -6264,7 +6264,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D79">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E79" t="str">
         <v>Occupied</v>
@@ -6284,7 +6284,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D80">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E80" t="str">
         <v>Occupied</v>
@@ -6304,7 +6304,7 @@
         <v>Penthouse</v>
       </c>
       <c r="D81">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="E81" t="str">
         <v>Occupied</v>
@@ -6732,7 +6732,7 @@
         <v>Complaints Filed</v>
       </c>
       <c r="B19">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20">
@@ -6796,7 +6796,7 @@
         <v>Seed Date</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-07-16T06:36:45.376Z</v>
+        <v>2026-08-07T04:30:50.544Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>